<commit_message>
Update 30-01-2026: Añadido cálculo tasas específicas AVP, AVD y AVAD
</commit_message>
<xml_diff>
--- a/datos_limpios/dic_arg_sim_avad_dm2.xlsx
+++ b/datos_limpios/dic_arg_sim_avad_dm2.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -516,7 +516,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Proyección poblacional por provincia, sexo y grupo etario decenal según Censo Nacional 2010</t>
+          <t>Proyección poblacional por sexo y grupo etario decenal según Censo Nacional 2010</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -533,12 +533,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>pob_est_2010</t>
+          <t>dm_total</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Población estándar por sexo y grupo etario decenal según Censo Nacional 2010</t>
+          <t>Total estimado de personas con diabetes mellitus (DM) por autorreporte según resultados ENFR</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -555,12 +555,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>dm_total</t>
+          <t>dm_total_se</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Total estimado de personas con diabetes mellitus (DM) por autorreporte según resultados ENFR</t>
+          <t>Error estándar del total estimado de personas con DM por autorreporte según resultados ENFR</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -577,12 +577,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dm_total_se</t>
+          <t>dm2_total</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Error estándar del total estimado de personas con DM por autorreporte según resultados ENFR</t>
+          <t>Total estimado de personas con DM tipo 2 (DM2) por autorreporte según resultados ENFR</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -599,12 +599,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>dm2_total</t>
+          <t>dm2_total_se</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Total estimado de personas con DM tipo 2 (DM2) por autorreporte según resultados ENFR</t>
+          <t>Error estándar del total estimado de personas con DM2 por autorreporte según resultados ENFR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -621,12 +621,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>dm2_total_se</t>
+          <t>dm2_prev</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Error estándar del total estimado de personas con DM2 por autorreporte según resultados ENFR</t>
+          <t>Prevalencia de personas con DM2 por autorreporte según resultados ENFR</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>dm2_prev</t>
+          <t>dm2_prev_se</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Prevalencia de personas con DM2 por autorreporte según resultados ENFR</t>
+          <t>Error estándar de la prevalencia de personas con DM2 por autorreporte según resultados ENFR</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -665,12 +665,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>dm2_prev_se</t>
+          <t>dm2_prev_cv</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Error estándar de la prevalencia de personas con DM2 por autorreporte según resultados ENFR</t>
+          <t>Coeficiente de variación de la prevalencia de personas con DM2 por autorreporte según resultados ENFR</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -687,12 +687,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>dm2_prev_cv</t>
+          <t>defun_n</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Coeficiente de variación de la prevalencia de personas con DM2 por autorreporte según resultados ENFR</t>
+          <t>Defunciones por DM2 para el trienio correspondiente a la ENFR</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -709,12 +709,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>defun_n</t>
+          <t>defun_mean</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Defunciones por DM2 para el trienio correspondiente a la ENFR</t>
+          <t>Defunciones promedio por DM2 para el trienio correspondiente a la ENFR</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -731,12 +731,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>defun_mean</t>
+          <t>defun_se</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Defunciones promedio por DM2 para el trienio correspondiente a la ENFR</t>
+          <t>Error estándar de las defunciones promedio por DM2 para el trienio correspondiente a la ENFR</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -753,12 +753,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>defun_se</t>
+          <t>ex</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Error estándar de las defunciones promedio por DM2 para el trienio correspondiente a la ENFR</t>
+          <t>Esperanza de vida a la edad X según sexo y grupo etario decenal</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -775,12 +775,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ex</t>
+          <t>fwd</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Esperanza de vida a la edad X según sexo y grupo etario decenal</t>
+          <t>Peso de discapacidad ponderado para secuelas de DM2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -797,12 +797,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>fwd</t>
+          <t>AVP</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Peso de discapacidad ponderado para secuelas de DM2</t>
+          <t>Años de vida perdidos (AVP) por muerte prematura por DM2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -819,12 +819,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AVP</t>
+          <t>AVP_inf</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Años de vida perdidos (AVP) por muerte prematura por DM2</t>
+          <t>Límite inferior del intervalo de incertidumbre (IU) de los AVP por muerte prematura por DM2</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -841,12 +841,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AVP_inf</t>
+          <t>AVP_sup</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Límite inferior del intervalo de incertidumbre (IU) de los AVP por muerte prematura por DM2</t>
+          <t>Límite superior del IU de los AVP por muerte prematura por DM2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -863,12 +863,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AVP_sup</t>
+          <t>AVD</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Límite superior del IU de los AVP por muerte prematura por DM2</t>
+          <t>Años vividos con discapacidad (AVD) por DM2</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -885,12 +885,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AVD</t>
+          <t>AVD_inf</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Años vividos con discapacidad (AVD) por DM2</t>
+          <t>Límite inferior del intervalo de incertidumbre (IU) de los AVD por DM2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -907,12 +907,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AVD_inf</t>
+          <t>AVD_sup</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Límite inferior del intervalo de incertidumbre (IU) de los AVD por DM2</t>
+          <t>Límite superior del IU de los AVD por DM2</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -929,12 +929,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AVD_sup</t>
+          <t>AVAD</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Límite superior del IU de los AVD por DM2</t>
+          <t>Años de vida ajustados por discapacidad (AVAD) para DM2</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -951,12 +951,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AVAD</t>
+          <t>AVAD_inf</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Años de vida ajustados por discapacidad (AVAD) para DM2</t>
+          <t>Límite inferior del intervalo de incertidumbre (IU) de los AVAD por DM2</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -973,12 +973,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AVAD_inf</t>
+          <t>AVAD_sup</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Límite inferior del intervalo de incertidumbre (IU) de los AVAD por DM2</t>
+          <t>Límite superior del IU de los AVAD por DM2</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -995,12 +995,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AVAD_sup</t>
+          <t>AVP_tasa</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Límite superior del IU de los AVAD por DM2</t>
+          <t>Tasa específica de AVP por DM2</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1009,6 +1009,182 @@
         </is>
       </c>
       <c r="D30" t="inlineStr">
+        <is>
+          <t>0-Inf</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>AVP_tasa_inf</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Límite inferior del intervalo de incertidumbre (IU) de la tasa de AVP por DM2</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>0-Inf</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>AVP_tasa_sup</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Límite superior del IU de la tasa de AVP por DM2</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>0-Inf</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>AVD_tasa</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Tasa específica de AVD por DM2</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>0-Inf</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>AVD_tasa_inf</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Límite inferior del intervalo de incertidumbre (IU) de la tasa de AVD por DM2</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>0-Inf</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>AVD_tasa_sup</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Límite superior del IU de la tasa de AVD por DM2</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>0-Inf</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>AVAD_tasa</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Tasa específica de AVAD por DM2</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>0-Inf</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>AVAD_tasa_inf</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Límite inferior del intervalo de incertidumbre (IU) de la tasa de AVAD por DM2</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>0-Inf</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>AVAD_tasa_sup</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Límite superior del IU de la tasa de AVAD por DM2</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
         <is>
           <t>0-Inf</t>
         </is>

</xml_diff>

<commit_message>
Update 30-01-2026: Añadido cálculo tasas específicas AVP, AVD y AVAD / Guardados datos como RDS para preservar formato
</commit_message>
<xml_diff>
--- a/datos_limpios/dic_arg_sim_avad_dm2.xlsx
+++ b/datos_limpios/dic_arg_sim_avad_dm2.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -533,12 +533,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>dm_total</t>
+          <t>pob_est_2010</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Total estimado de personas con diabetes mellitus (DM) por autorreporte según resultados ENFR</t>
+          <t>Población estándar por sexo y grupo etario decenal según Censo Nacional 2010</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -555,12 +555,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>dm_total_se</t>
+          <t>dm_total</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Error estándar del total estimado de personas con DM por autorreporte según resultados ENFR</t>
+          <t>Total estimado de personas con diabetes mellitus (DM) por autorreporte según resultados ENFR</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -577,12 +577,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dm2_total</t>
+          <t>dm_total_se</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Total estimado de personas con DM tipo 2 (DM2) por autorreporte según resultados ENFR</t>
+          <t>Error estándar del total estimado de personas con DM por autorreporte según resultados ENFR</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -599,12 +599,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>dm2_total_se</t>
+          <t>dm2_total</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Error estándar del total estimado de personas con DM2 por autorreporte según resultados ENFR</t>
+          <t>Total estimado de personas con DM tipo 2 (DM2) por autorreporte según resultados ENFR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -621,12 +621,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>dm2_prev</t>
+          <t>dm2_total_se</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Prevalencia de personas con DM2 por autorreporte según resultados ENFR</t>
+          <t>Error estándar del total estimado de personas con DM2 por autorreporte según resultados ENFR</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>dm2_prev_se</t>
+          <t>dm2_prev</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Error estándar de la prevalencia de personas con DM2 por autorreporte según resultados ENFR</t>
+          <t>Prevalencia de personas con DM2 por autorreporte según resultados ENFR</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -665,12 +665,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>dm2_prev_cv</t>
+          <t>dm2_prev_low</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Coeficiente de variación de la prevalencia de personas con DM2 por autorreporte según resultados ENFR</t>
+          <t>Límite inferior del intervalo de confianza (CI) de la prevalencia de personas con DM2 por autorreporte según resultados ENFR</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -687,12 +687,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>defun_n</t>
+          <t>dm2_prev_upp</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Defunciones por DM2 para el trienio correspondiente a la ENFR</t>
+          <t>Límite superior del intervalo de confianza (CI) de la prevalencia de personas con DM2 por autorreporte según resultados ENFR</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -709,12 +709,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>defun_mean</t>
+          <t>dm2_prev_cv</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Defunciones promedio por DM2 para el trienio correspondiente a la ENFR</t>
+          <t>Coeficiente de variación de la prevalencia de personas con DM2 por autorreporte según resultados ENFR</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -731,12 +731,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>defun_se</t>
+          <t>defun_n</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Error estándar de las defunciones promedio por DM2 para el trienio correspondiente a la ENFR</t>
+          <t>Defunciones por DM2 para el trienio correspondiente a la ENFR</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -753,12 +753,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ex</t>
+          <t>defun_mean</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Esperanza de vida a la edad X según sexo y grupo etario decenal</t>
+          <t>Defunciones promedio por DM2 para el trienio correspondiente a la ENFR</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -775,12 +775,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>fwd</t>
+          <t>defun_se</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Peso de discapacidad ponderado para secuelas de DM2</t>
+          <t>Error estándar de las defunciones promedio por DM2 para el trienio correspondiente a la ENFR</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -797,12 +797,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AVP</t>
+          <t>ex</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Años de vida perdidos (AVP) por muerte prematura por DM2</t>
+          <t>Esperanza de vida a la edad X según sexo y grupo etario decenal</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -819,12 +819,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AVP_inf</t>
+          <t>fwd</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Límite inferior del intervalo de incertidumbre (IU) de los AVP por muerte prematura por DM2</t>
+          <t>Peso de discapacidad ponderado para secuelas de DM2</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -841,12 +841,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AVP_sup</t>
+          <t>AVP</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Límite superior del IU de los AVP por muerte prematura por DM2</t>
+          <t>Años de vida perdidos (AVP) por muerte prematura por DM2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -863,12 +863,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AVD</t>
+          <t>AVP_low</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Años vividos con discapacidad (AVD) por DM2</t>
+          <t>Límite inferior del intervalo de incertidumbre (IU) de los AVP por muerte prematura por DM2</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -885,12 +885,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AVD_inf</t>
+          <t>AVP_upp</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Límite inferior del intervalo de incertidumbre (IU) de los AVD por DM2</t>
+          <t>Límite superior del IU de los AVP por muerte prematura por DM2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -907,12 +907,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AVD_sup</t>
+          <t>AVD</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Límite superior del IU de los AVD por DM2</t>
+          <t>Años vividos con discapacidad (AVD) por DM2</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -929,12 +929,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AVAD</t>
+          <t>AVD_low</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Años de vida ajustados por discapacidad (AVAD) para DM2</t>
+          <t>Límite inferior del intervalo de incertidumbre (IU) de los AVD por DM2</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -951,12 +951,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AVAD_inf</t>
+          <t>AVD_upp</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Límite inferior del intervalo de incertidumbre (IU) de los AVAD por DM2</t>
+          <t>Límite superior del IU de los AVD por DM2</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -973,12 +973,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AVAD_sup</t>
+          <t>AVAD</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Límite superior del IU de los AVAD por DM2</t>
+          <t>Años de vida ajustados por discapacidad (AVAD) para DM2</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -995,12 +995,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AVP_tasa</t>
+          <t>AVAD_low</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Tasa específica de AVP por DM2</t>
+          <t>Límite inferior del intervalo de incertidumbre (IU) de los AVAD por DM2</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1017,12 +1017,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>AVP_tasa_inf</t>
+          <t>AVAD_upp</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Límite inferior del intervalo de incertidumbre (IU) de la tasa de AVP por DM2</t>
+          <t>Límite superior del IU de los AVAD por DM2</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1039,12 +1039,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AVP_tasa_sup</t>
+          <t>AVP_tasa</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Límite superior del IU de la tasa de AVP por DM2</t>
+          <t>Tasa específica de AVP por DM2</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1061,12 +1061,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AVD_tasa</t>
+          <t>AVP_tasa_low</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Tasa específica de AVD por DM2</t>
+          <t>Límite inferior del intervalo de incertidumbre (IU) de la tasa de AVP por DM2</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1083,12 +1083,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>AVD_tasa_inf</t>
+          <t>AVP_tasa_upp</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Límite inferior del intervalo de incertidumbre (IU) de la tasa de AVD por DM2</t>
+          <t>Límite superior del IU de la tasa de AVP por DM2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1105,12 +1105,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AVD_tasa_sup</t>
+          <t>AVD_tasa</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Límite superior del IU de la tasa de AVD por DM2</t>
+          <t>Tasa específica de AVD por DM2</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1127,12 +1127,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AVAD_tasa</t>
+          <t>AVD_tasa_low</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Tasa específica de AVAD por DM2</t>
+          <t>Límite inferior del intervalo de incertidumbre (IU) de la tasa de AVD por DM2</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1149,12 +1149,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>AVAD_tasa_inf</t>
+          <t>AVD_tasa_upp</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Límite inferior del intervalo de incertidumbre (IU) de la tasa de AVAD por DM2</t>
+          <t>Límite superior del IU de la tasa de AVD por DM2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1171,20 +1171,64 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>AVAD_tasa_sup</t>
+          <t>AVAD_tasa</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>Tasa específica de AVAD por DM2</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>0-Inf</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>AVAD_tasa_low</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Límite inferior del intervalo de incertidumbre (IU) de la tasa de AVAD por DM2</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>0-Inf</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>AVAD_tasa_upp</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
           <t>Límite superior del IU de la tasa de AVAD por DM2</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>numeric</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
         <is>
           <t>0-Inf</t>
         </is>

</xml_diff>